<commit_message>
260307016EA maps: study limits and the circled fatal crash on the AADT map, 2023 median year
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UzM4sZHfA2PkELFhftQzNK
</commit_message>
<xml_diff>
--- a/examples/260307016EA/260307016EA_CalculatedAADT.xlsx
+++ b/examples/260307016EA/260307016EA_CalculatedAADT.xlsx
@@ -511,9 +511,8 @@
           <t>Median Year:</t>
         </is>
       </c>
-      <c r="F4" s="1">
-        <f>(B3+B4)/2</f>
-        <v/>
+      <c r="F4" t="n">
+        <v>2023</v>
       </c>
     </row>
     <row r="5">
@@ -601,7 +600,7 @@
         <v>4400</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="E11" s="5">
         <f>C11*(1+$B$5)</f>
@@ -625,10 +624,10 @@
         <v>0.542</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>4400</v>
+        <v>4500</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="E12" s="5">
         <f>C12*(1+$B$5)</f>
@@ -1180,7 +1179,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Study period 8/1/2021 to 7/31/2026; the median year falls in early 2024, so the 2024 AADT is used for each section.</t>
+          <t>Study period 8/1/2021 to 7/31/2026. 2023 is the median year used for the analysis, so the 2023 AADT is used for each section.</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1214,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>The TEAAS strip analysis used ADT 4400 (route 30000311 in the study criteria); the calculated ADT matches, so the study ADT is kept.</t>
+          <t>The TEAAS strip analysis used ADT 4400 (route 30000311 in the study criteria). The calculated ADT rounds to 4400 and the difference is about 1 percent, so the study ADT is kept.</t>
         </is>
       </c>
     </row>

</xml_diff>